<commit_message>
Fixed Download Error Message Bug; revised Test Script; added BERT Score
</commit_message>
<xml_diff>
--- a/Model_Testing/Questions.xlsx
+++ b/Model_Testing/Questions.xlsx
@@ -49,7 +49,7 @@
     <t xml:space="preserve">Where is the city of Cologne located?</t>
   </si>
   <si>
-    <t xml:space="preserve">The city of Cologne is Köln, and it is located in the district Köln, the administrative district Köln, and the federal state of Nordrhein-Westfalen.</t>
+    <t xml:space="preserve">The city of Cologne is located in the administrative district Köln, and the federal state of Nordrhein-Westfalen.</t>
   </si>
   <si>
     <t xml:space="preserve">Where is the administrative community of Eisenhüttenstadt located?</t>
@@ -67,7 +67,7 @@
     <t xml:space="preserve">Where is the district of Gießen located?</t>
   </si>
   <si>
-    <t xml:space="preserve">The district of Gießen is located in Gießen, which is in Hessen. The hierarchy levels are: District Gießen, and FederalState Hessen.</t>
+    <t xml:space="preserve">The district of Gießen is located in the federal state of Hessen.</t>
   </si>
   <si>
     <t xml:space="preserve">Where is the district of Nordsachsen located?</t>
@@ -79,7 +79,7 @@
     <t xml:space="preserve">Where is the administrative district of Freiburg located?</t>
   </si>
   <si>
-    <t xml:space="preserve">The AdministrativeDistrict Freiburg is located in the FederalState Baden-Württemberg.</t>
+    <t xml:space="preserve">The administrative district Freiburg is located in the federalstate Baden-Württemberg.</t>
   </si>
   <si>
     <t xml:space="preserve">Where is the administrative district of Oberfranken located?</t>
@@ -91,34 +91,34 @@
     <t xml:space="preserve">Where is the federal state of Sachsen located?</t>
   </si>
   <si>
-    <t xml:space="preserve">The federal state of Sachsen is located at POINT (13.348518008906732 51.05230081187263).</t>
+    <t xml:space="preserve">The federal state of Sachsen is located at the federalstate level. The centroid coordinates for Sachen are at POINT (13.348518008906732 51.05230081187263).</t>
   </si>
   <si>
     <t xml:space="preserve">Where is the federal state of Saarland located?</t>
   </si>
   <si>
-    <t xml:space="preserve">The federal state Saarland is located at the FederalState level.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">physical/parts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which cities are part of the District of Coesfeld?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The District of Coesfeld includes the cities of Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, and Ascheberg.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which Districts are located within the Administrative District of Oberbayern?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Administrative District of Oberbayern includes the following Districts: Fürstenfeldbruck, Erding, München, Freising, Ingolstadt, Mühldorf a.Inn, Rosenheim, Garmisch-Partenkirchen, Eichstätt, Landsberg am Lech, Weilheim-Schongau, Dachau, Altötting, Neuburg-Schrobenhausen, Pfaffenhofen a.d.Ilm, Ebersberg, Bad Tölz-Wolfratshausen, Traunstein, Miesbach, Starnberg, and Berchtesgadener Land. It also includes more than one District named Rosenheim and more than one District named München.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which Districts belong to the Federal State of Hessen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Federal State of Hessen includes the following districts: Offenbach am Main, Groß-Gerau, Main-Taunus-Kreis, Wetteraukreis, Offenbach, Main-Kinzig-Kreis, Hochtaunuskreis, Odenwaldkreis, Darmstadt-Dieburg, Rheingau-Taunus-Kreis, Wiesbaden, Frankfurt am Main, Bergstraße, Darmstadt, Marburg-Biedenkopf, Gießen, Lahn-Dill-Kreis, Limburg-Weilburg, Vogelsbergkreis, Schwalm-Eder-Kreis, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, and Hersfeld-Rotenburg.</t>
+    <t xml:space="preserve">The federal state Saarland is located at the federalstate level. The centroid coordinates for Saarland at POINT (6.953360955673903 49.38438040655551).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">physical/parts - enumeration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which cities are part of the district of Coesfeld?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The district of Coesfeld includes the cities of Coesfeld, Olfen, Senden, Nottuln, Havixbeck, Nordkirchen, Billerbeck, Lüdinghausen, Rosendahl, Dülmen, and Ascheberg.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which districts are located within the administrative district of Oberbayern?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The administrative district of Oberbayern includes the following districts: Fürstenfeldbruck, Erding, München, Freising, Ingolstadt, Mühldorf a.Inn, Rosenheim, Garmisch-Partenkirchen, Eichstätt, Landsberg am Lech, Weilheim-Schongau, Dachau, Altötting, Neuburg-Schrobenhausen, Pfaffenhofen a.d.Ilm, Ebersberg, Bad Tölz-Wolfratshausen, Traunstein, Miesbach, Starnberg, and Berchtesgadener Land. It also includes more than one district named Rosenheim and more than one district named München.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which districts belong to the federal state of Hessen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The federal state of Hessen includes the following districts: Offenbach am Main, Groß-Gerau, Main-Taunus-Kreis, Wetteraukreis, Offenbach, Main-Kinzig-Kreis, Hochtaunuskreis, Odenwaldkreis, Darmstadt-Dieburg, Rheingau-Taunus-Kreis, Wiesbaden, Frankfurt am Main, Bergstraße, Darmstadt, Marburg-Biedenkopf, Gießen, Lahn-Dill-Kreis, Limburg-Weilburg, Vogelsbergkreis, Schwalm-Eder-Kreis, Kassel, Waldeck-Frankenberg, Fulda, Werra-Meißner-Kreis, and Hersfeld-Rotenburg.</t>
   </si>
   <si>
     <t xml:space="preserve">Which administrative communities has the district of Steinburg?</t>
@@ -130,34 +130,34 @@
     <t xml:space="preserve">How many cities belong to the district of Paderborn?</t>
   </si>
   <si>
-    <t xml:space="preserve">The District of Paderborn includes 10 cities: Paderborn, Bad Lippspringe, Borchen, Büren, Altenbeken, Hövelhof, Lichtenau, Bad Wünnenberg, Salzkotten, and Delbrück.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">physical/parts decision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Does the city of Dülmen lie within the District of Coesfeld?</t>
+    <t xml:space="preserve">The district of Paderborn includes 10 cities: Paderborn, Bad Lippspringe, Borchen, Büren, Altenbeken, Hövelhof, Lichtenau, Bad Wünnenberg, Salzkotten, and Delbrück.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">physical/parts - comparison</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the city of Dülmen lie within the district of Coesfeld?</t>
   </si>
   <si>
     <t xml:space="preserve">Yes. Dülmen, a city, lies within Coesfeld, a district.</t>
   </si>
   <si>
-    <t xml:space="preserve">Is the District of Coesfeld located in the Administrative District of Münster?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes, the District of Coesfeld is located in the Administrative District of Münster.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Does the Administrative District of Oberfranken belong to the Federal State of Bayern?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes, the Administrative District of Oberfranken belongs to the Federal State of Bayern. The Administrative District is Oberfranken, and the Federal State is Bayern.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is the District of Steinfurt located in the Federal State of Nordrhein-Westfalen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes, the District of Steinfurt is located in the Federal State of Nordrhein-Westfalen.</t>
+    <t xml:space="preserve">Is the district of Coesfeld located in the administrative district of Münster?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, the district of Coesfeld is located in the administrative district of Münster.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Does the administrative district of Oberfranken belong to the federal state of Bayern?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, the administrative district of Oberfranken belongs to the federal state of Bayern.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Is the district of Steinfurt located in the federal state of Nordrhein-Westfalen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, the district of Steinfurt is located in the federal state of Nordrhein-Westfalen.</t>
   </si>
   <si>
     <t xml:space="preserve">Is the city of Bocholt located within the district of Cloppenburg?</t>
@@ -169,10 +169,10 @@
     <t xml:space="preserve">topological (1:1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Do the Districts of Coesfeld and Borken touch each other?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes, the District of Coesfeld and the District of Borken touch each other.</t>
+    <t xml:space="preserve">Do the districts of Coesfeld and Borken touch each other?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, the district of Coesfeld and the district of Borken touch each other.</t>
   </si>
   <si>
     <t xml:space="preserve">Are the cities of Senden and Münster geographically disjoint?</t>
@@ -181,16 +181,16 @@
     <t xml:space="preserve">No. Senden and Münster are next to each other.</t>
   </si>
   <si>
-    <t xml:space="preserve">Does the Federal State of Niedersachsen touch Nordrhein-Westfalen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yes, the Federal State Niedersachsen touches the Federal State Nordrhein-Westfalen.</t>
+    <t xml:space="preserve">Does the federal state of Niedersachsen touch Nordrhein-Westfalen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, the federal state Niedersachsen touches the federal state Nordrhein-Westfalen.</t>
   </si>
   <si>
     <t xml:space="preserve">Is Berlin completely surrounded by Brandenburg?</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes.</t>
+    <t xml:space="preserve">Yes, Berlin is surrounded by Brandenburg.</t>
   </si>
   <si>
     <t xml:space="preserve">cardinal (1:1)</t>
@@ -199,19 +199,19 @@
     <t xml:space="preserve">Is Münster north of Dortmund?</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes, Münster is north of Dortmund. The place Dortmund is a City, and Münster is also a City.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which city is located directly north of Jever?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wangerland is located directly north of Jever.</t>
+    <t xml:space="preserve">Yes, Münster is north of Dortmund.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which city is located directly north of Münster?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greven is located directly north of Münster.</t>
   </si>
   <si>
     <t xml:space="preserve">Is Leipzig located northeast of Erfurt?</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes. Leipzig is located northeast of Erfurt.</t>
+    <t xml:space="preserve">Yes, Leipzig is located northeast of Erfurt.</t>
   </si>
   <si>
     <t xml:space="preserve">distance (1:1)</t>
@@ -220,19 +220,19 @@
     <t xml:space="preserve">What is the distance between the cities of Köln and Bonn?</t>
   </si>
   <si>
-    <t xml:space="preserve">The distance between the City of Köln and the City of Bonn is 6.63 km.</t>
+    <t xml:space="preserve">The distance between the city of Köln and the city of Bonn is 6.63 km.</t>
   </si>
   <si>
     <t xml:space="preserve">How far is it from Hannover to Braunschweig?</t>
   </si>
   <si>
-    <t xml:space="preserve">The distance from the City of Hannover to the City of Braunschweig is 34.92 km.</t>
+    <t xml:space="preserve">The distance from the city of Hannover to the city of Braunschweig is 34.92 km.</t>
   </si>
   <si>
     <t xml:space="preserve">How far are Hessen and Thüringen from each other?</t>
   </si>
   <si>
-    <t xml:space="preserve">Hessen and Thüringen, both FederalStates, are 0.0 km apart.</t>
+    <t xml:space="preserve">Hessen and Thüringen, both federalstates, are 0.0 km apart.</t>
   </si>
   <si>
     <t xml:space="preserve">topological (1:N)</t>
@@ -241,69 +241,67 @@
     <t xml:space="preserve">Which are the three closest districts to the district of Miesbach?</t>
   </si>
   <si>
-    <t xml:space="preserve">The three closest Districts to the District of Miesbach are Bad Tölz-Wolfratshausen, München, and Rosenheim.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which Districts touch the District of Warendorf?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The District of Warendorf touches the Districts of Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, and Soest.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which administrative communities are adjacent to Leezen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The administrative communities adjacent to Leezen are Groß Niendorf, Mözen, Kükels, Fredesdorf, Seth, Sülfeld, Neversdorf, and Bebensee. Leezen is also adjacent to Langen Brütz, Lübstorf, Raben Steinfeld, Cambs, Dobin am See, Schwerin, Gneven, and Pinnow.
-There are two places named Leezen in different City levels, so the answer refers to both City &lt; AdministrativeCommunity &lt; District &lt; AdministrativeDistrict &lt; FederalState hierarchy contexts.</t>
+    <t xml:space="preserve">The three closest districts to the district of Miesbach are Bad Tölz-Wolfratshausen, München, and Rosenheim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which districts touch the district of Warendorf?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The district of Warendorf touches the districts of Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld, and Soest.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which administrative communities are adjacent to the administrative community Leezen? </t>
+  </si>
+  <si>
+    <t xml:space="preserve">The administrative community Leezen is adjacent to these administrative communities: Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling, and Buchholz (Forstgutsbez.). </t>
   </si>
   <si>
     <t xml:space="preserve">By which administrative districts is Mittelfranken surrounded?</t>
   </si>
   <si>
-    <t xml:space="preserve">Mittelfranken, an AdministrativeDistrict, is surrounded by Bayern, a FederalState.</t>
+    <t xml:space="preserve">Mittelfranken is surrounded by the administrative districts of Oberpfalz, Unterfranken, Oberfranken, Oberbayern, Schwaben, and Stuttgart.</t>
   </si>
   <si>
     <t xml:space="preserve">cardinal (1:N)</t>
   </si>
   <si>
-    <t xml:space="preserve">Which Federal States are located north of Thüringen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The Federal State Thüringen is associated with Hamburg, Schleswig-Holstein, Mecklenburg-Vorpommern, Thüringen, and Sachsen-Anhalt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which Districts are west of the district of Münster?</t>
+    <t xml:space="preserve">Which federal states are located north of Thüringen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The federal states north of Thüringen are Hamburg, Schleswig-Holstein, Mecklenburg-Vorpommern, and Sachsen-Anhalt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which districts are west of the district of Münster?</t>
   </si>
   <si>
     <t xml:space="preserve">The districts Kleve and Borken are west of Münster.</t>
   </si>
   <si>
-    <t xml:space="preserve">Which administrative communities are located north of the administrative community Morbach?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The administrative communities located north of Morbach are Emlichheim, Viöl, Osterholz-Scharmbeck, Kappeln-Land, Wilster, Vordereifel, Wangerland, Ovelgönne, Schortens, Wangerooge, Südtondern, Brookmerland, Kellinghusen, Cappeln (Oldenburg), Wagenfeld, Mittelholstein, Rendsburg, Wietmarschen, Georgsmarienhütte, Hasbergen, Pinneberg, Marne-Nordsee, Rengsdorf-Waldbreitbach, Bokhorst-Wankendorf, Rantzau, Mittleres Nordfriesland, Hamm (Sieg), Südbrookmerland, Tornesch, Selsingen, Esens, Langeoog, Drochtersen, Glandorf, Elmshorn-Land, Steinfeld (Oldenburg), Lengerich, Steyerberg, Aurich, Bohmte, Bönebüttel, Butjadingen, Geeste, Wasbek, Rehden, Apensen, Stadland, Damme, Bad Essen, Westerstede, Schlei-Ostsee, Westoverledingen, Bad Bentheim, Langballig, Bad Hönningen, Weyhe, Eidertal, Werlte, Elmshorn, Bunde, Horst-Herzhorn, Brunsbüttel, Ihlow, Barßel, Bakum, Garrel, Artland, Tarmstedt, Jever, Landschaft Sylt, Arensharde, Nordhorn, Gnarrenburg, Eiderkanal, Holdorf, Insel Lütje Hörn, Husum, Eiderstedt, Kappeln, Schüttorf, Zell (Mosel), Altenahr, Sylt, Ritterhude, Süderbrarup, Neuenkirchen, Hesel, Wildeshausen, Dänischenhagen, Wurster Nordseeküste, Emsbüren, Fockbek, Vechta, Berne, Nordsee-Treene, Bruchhausen-Vilsen, Kirchspielslandgemeinden Eider, Cochem, Hagen am Teutoburger Wald, Mittelangeln, Hohner Harde, Uelsen, Twistringen, Bramsche, Bad Neuenahr-Ahrweiler, Herzlake, Rhede (Ems), Schrevenborn, Stade, Schwanewede, Wittmund, Borkum, Bad Zwischenahn, Sittensen, Sulingen, Heide, Dötlingen, Glücksburg (Ostsee), Schleswig, Weener, Oeversee, Mendig, Salzbergen, Nordenham, Handewitt, Südangeln, Pinnau, Pellworm, Cuxhaven, Uplengen, Geestequelle, Ottersberg, Kirchdorf, Dinklage, Puderbach, Breitenburg, Nordhümmling, Jümme, Rhauderfehn, Rotenburg (Wümme), Maifeld, Hage, Zeven, Haren (Ems), Sande, Preetz-Land, Wardenburg, Syke, Eggebek, Langwedel, Grafschaft Hoya, Schwentinental, Lemwerder, Jemgum, Barmstedt, Fürstenau, Juist, Visbek, Oldenburg (Oldb), Burg-St. Michaelisdonn, Beverstedt, Lathen, Meppen, Geltinger Bucht, Hilter am Teutoburger Wald, Altenkirchen-Flammersfeld, Lilienthal, Rastede, Adenau, Auenland Südholstein, Uchte, Bissendorf, Flensburg, Kiel, Grasberg, Mitteldithmarschen, Hörnerkirchen, Wiesmoor, Bad Laer, Kaltenkirchen, Altes Amt Lemförde, Barnstorf, Elsfleth, Ostrhauderfehn, Harpstedt, Hatten, Itzehoe, Belm, Bersenbrück, Helgoland, Schenefeld, Neuwied, Andernach, Oldendorf-Himmelpforten, Oyten, Itzehoe-Land, Harrislee, Norden, Kirchspielslandgemeinde Heider Umland, Asbach, Melle, Sögel, Kropp-Stapelholm, Haddeby, Papenburg, Apen, Reußenköge, Fredenbeck, Kelberg, Achterwehr, Siedenburg, Spiekeroog, Bad Rothenfelde, Zetel, Remagen, Baltrum, Neuenkirchen-Vörden, Uetersen, Cloppenburg, Schiffdorf, Linz am Rhein, Leer (Ostfriesland), Wilstermarsch, Ulmen, Dissen am Teutoburger Wald, Schwaförden, Moormerland, Hürup, Emden, Mayen, Großefehn, Unkel, Worpswede, Sinzig, Bösel, Harsefeld, Neumünster, Neuenhaus, Jade, Bad Breisig, Friedrichstadt, Friesoythe, Jork, Hagen im Bremischen, Holtriem, Verden (Aller), Probstei, Lastrup, Sottrum, Lindern (Oldenburg), Ostercappeln, Bad Bramstedt, Dornum, Goldenstedt, Lingen (Ems), Freren, Emstek, Börde Lamstedt, Essen (Oldenburg), Geest und Marsch Südholstein, Schafflund, Bordesholm, Nordseeinsel Memmert, Dänischer Wohld, Saterland, Nortorfer Land, Bockhorn, Geestland, Molbergen, Jevenstedt, Loxstedt, Büdelsdorf, Föhr-Amrum, Krummhörn, Dörpen, Norderney, Bremervörde, Bad Bramstedt-Land, Stuhr, Wilhelmshaven, Tönning, Hemmoor, Haselünne, Wallenhorst, Thedinghausen, Kaisersesch, Kronshagen, Großheide, Friedeburg, Lühe, Brake (Unterweser), Bad Iburg, Traben-Trarbach, Brohltal, Löningen, Grafschaft, Twist, Eckernförde, Pellenz, Ganderkesee, Großenkneten, Krempermarsch, Diepholz, Nordkehdingen, Hude (Oldb), Varel, Altenholz, Delmenhorst, Büsum-Wesselburen, Osnabrück, Hinte, Hambergen, Glückstadt, Wedel, Bassum, Horneburg, Edewecht, Hüttener Berge, Achim, Wiefelstede, Lohne (Oldenburg), Spelle, and Land Hadeln.</t>
+    <t xml:space="preserve">Which administrative communities are located north of the administrative community Kiel?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The administrative communities located north of the administrative community Kiel are: Altenholz, Dänischenhagen, Kappeln and Geltinger Bucht.</t>
   </si>
   <si>
     <t xml:space="preserve">distance (1:N)</t>
   </si>
   <si>
-    <t xml:space="preserve">Which Districts are located within a radius of 10 km from the district Göttingen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The District Göttingen is located within a radius of 10 km from the following Districts: Eichsfeld, Werra-Meißner-Kreis, Harz, Kassel, Goslar, Northeim, Nordhausen, and Kassel.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which cities are located in a radius of 15 km of Aachen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Within a radius of 15 km around the City Aachen, the following Cities are located: Stolberg (Rhld.), Aldenhoven, Roetgen, Gangelt, Nideggen, Inden, Eschweiler, Heimbach, Baesweiler, Alsdorf, Linnich, Würselen, Langerwehe, Monschau, Hürtgenwald, Kreuzau, Düren, Jülich, Simmerath, Geilenkirchen, Übach-Palenberg, and Herzogenrath.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Which cities are located less than 20 km around Munich?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The cities and places located less than 20 km around Munich are: Haar, Forstenrieder Park, Unterföhring, Bergkirchen, Berg, Markt Schwaben, Weichs, Wörth, Starnberg, Neuried, Mammendorf, Sulzemoos, Moorenweis, Hohenkammer, Schöngeising, Schwabhausen, Hohenlinden, Olching, Marzling, Allershausen, Grünwald, Weßling, Alling, Planegg, Putzbrunn, Odelzhausen, Eglhartinger Forst, Oberschleißheim, Poing, Landsberied, Taufkirchen, Vaterstetten, Forstern, Inning a.Ammersee, Wolfratshausen, Münsing, Andechs, Grafrath, Finsing, Kirchseeon, Wörthsee, Petershausen, Fahrenzhausen, Schäftlarn, Krailling, Aschheim, Altomünster, Maisach, Egmating, Karlsfeld, Ebersberg, Ottobrunn, Aying, Röhrmoos, Zorneding, Unterhaching, Haimhausen, Neuching, Kottgeisering, Oberhaching, Erding, Adelshofen, Althegnenberg, Eching am Ammersee, Ismaning, Brunnthal, Forstinning, Walpertskirchen, Bruck, Gröbenzell, Freising, Baierbrunn, Türkenfeld, Egling, Oberding, Aßling, Kirchheim b.München, Garching b.München, Emmering, Otterfing, Germering, Neubiberg, Pliening, Baiern, Eching, Ebersberger Forst, Valley, Kranzberg, Icking, Pfaffenhofen a.d.Glonn, Anzinger Forst, Markt Indersdorf, Vierkirchen, Feldkirchen-Westerham, Jetzendorf, Fürstenfeldbruck, Moosinning, Feldkirchen, Grünwalder Forst, Hallbergmoos, Geretsried, Ammersee, Hebertshausen, Wolfratshauser Forst, Dietramszell, Egenhofen, Starnberger See, Unterschleißheim, Gauting, Neufahrn b.Freising, Straßlach-Dingharting, Perlacher Forst, Höhenkirchen-Siegertsbrunn, Moosach, Dachau, Hattenhofen, Grafing b.München, Pullach i.Isartal, Grasbrunn, Oberpframmern, Ottenhofen, Gilching, Anzing, Pöcking, Mittelstetten, Erdweg, Glonn, Gräfelfing, Holzkirchen, Pupplinger Au, Feldafing, Jesenwang, Pastetten, Sauerlach, Eichenau, Oberschweinbach, Weyarn, Seefeld, Puchheim, Hohenbrunn, and Herrsching a.Ammersee.
-They are all given as City entities around München, which is the City being queried.</t>
+    <t xml:space="preserve">Which districts are located within a radius of 10 km from the district Göttingen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The district Göttingen has the following districts within a radius of 10 km: Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis, and Nordhausen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which cities are located in a radius of 5 km of Aachen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The following cities are located within a radius of 5 km of Aachen: Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen,  Herzogenrath, Eschweiler, Stolberg (Rhld.).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Which cities are located less than 2 km around Munich?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The cities located less than 2 km around Munich are: Forstenrieder Park, Grünwald, Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i.Isartal, Bergkirchen, Neuried, Germering, Olching, Garching b.München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing, and Karlsfeld. </t>
   </si>
   <si>
     <t xml:space="preserve">DE</t>
@@ -318,7 +316,7 @@
     <t xml:space="preserve">Wo liegt die Stadt Köln?</t>
   </si>
   <si>
-    <t xml:space="preserve">Die Stadt Köln heißt Köln und liegt im Bezirk Köln, im Regierungsbezirk Köln und im Bundesland Nordrhein-Westfalen.</t>
+    <t xml:space="preserve">Die Stadt Köln liegt im Regierungsbezirk Köln und im Bundesland Nordrhein-Westfalen.</t>
   </si>
   <si>
     <t xml:space="preserve">Wo liegt die Verwaltungsgemeinschaft Eisenhüttenstadt?</t>
@@ -336,7 +334,7 @@
     <t xml:space="preserve">Wo liegt der Kreis Gießen?</t>
   </si>
   <si>
-    <t xml:space="preserve">Der Landkreis Gießen liegt in Gießen, das in Hessen liegt. Die Hierarchieebenen sind: Landkreis Gießen und Bundesland Hessen.</t>
+    <t xml:space="preserve">Der Landkreis Gießen liegt im Bundesland Hessen.</t>
   </si>
   <si>
     <t xml:space="preserve">Wo liegt der Kreis Nordsachsen?</t>
@@ -360,13 +358,13 @@
     <t xml:space="preserve">Wo liegt das Bundesland Sachsen?</t>
   </si>
   <si>
-    <t xml:space="preserve">Das Bundesland Sachsen befindet sich auf Bundeslandsebene.</t>
+    <t xml:space="preserve">Sachsen liegt auf Bundeslandebene beim Punkt  (13.348518008906732 51.05230081187263).</t>
   </si>
   <si>
     <t xml:space="preserve">Wo liegt das Bundesland Saarland?</t>
   </si>
   <si>
-    <t xml:space="preserve">Das Bundesland Saarland befindet sich auf Bundeslandsebene.</t>
+    <t xml:space="preserve">Das Saarland liegt auf Bundeslandebene beim Punkt (6,953360955673903 49,38438040655551).</t>
   </si>
   <si>
     <t xml:space="preserve">Welche Städte gehören zum Kreis Coesfeld?</t>
@@ -414,7 +412,7 @@
     <t xml:space="preserve">Gehört der Regierungsbezirk Oberfranken zum Bundesland Bayern?</t>
   </si>
   <si>
-    <t xml:space="preserve">Ja, der Regierungsbezirk Oberfranken gehört zum Bundesland Bayern. Der Regierungsbezirk ist Oberfranken, das Bundesland ist Bayern.</t>
+    <t xml:space="preserve">Ja, der Regierungsbezirk Oberfranken gehört zum Bundesland Bayern.</t>
   </si>
   <si>
     <t xml:space="preserve">Befindet sich der Kreis Steinfurt im Bundesland Nordrhein-Westfalen?</t>
@@ -450,25 +448,25 @@
     <t xml:space="preserve">Ist Berlin vollständig von Brandenburg umgeben?</t>
   </si>
   <si>
-    <t xml:space="preserve">Ja.</t>
+    <t xml:space="preserve">Ja, Berlin ist von Brandenburg umgeben.</t>
   </si>
   <si>
     <t xml:space="preserve">Liegt Münster nördlich von Dortmund?</t>
   </si>
   <si>
-    <t xml:space="preserve">Ja, Münster liegt nördlich von Dortmund. Dortmund ist eine Stadt, und Münster ist ebenfalls eine Stadt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welche Stadt liegt direkt nördlich von Jever?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wangerland liegt direkt nördlich von Jever.</t>
+    <t xml:space="preserve">Ja, Münster liegt nördlich von Dortmund.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welche Stadt liegt direkt nördlich von Münster?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Greven liegt direkt nördlich von Münster.</t>
   </si>
   <si>
     <t xml:space="preserve">Liegt Leipzig östlich von Erfurt?</t>
   </si>
   <si>
-    <t xml:space="preserve">Ja. Leipzig liegt nordöstlich von Erfurt.</t>
+    <t xml:space="preserve">Ja, Leipzig liegt nordöstlich von Erfurt.</t>
   </si>
   <si>
     <t xml:space="preserve">Wie groß ist die Entfernung zwischen den Städten Köln und Bonn?</t>
@@ -501,10 +499,10 @@
     <t xml:space="preserve">Der Kreis Warendorf grenzt an die Kreise Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld und Soest.</t>
   </si>
   <si>
-    <t xml:space="preserve">Welche Verwaltungsgemeinschaften grenzen an Leezen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Es gibt zwei Orte namens Leezen auf unterschiedlichen Verwaltungsebenen, daher bezieht sich die Antwort auf beide Hierarchiekontexte: Stadt &lt; Gemeinde &lt; Kreis &lt; Verwaltungsbezirk &lt; Bundesland.“</t>
+    <t xml:space="preserve">Welche Verwaltungsbezirke grenzen an den Verwaltungsbezirk Leezen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Verwaltungsbezirk Leezen grenzt an folgende Verwaltungsbezirke: Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling und Buchholz (Forstgutsbezirk).</t>
   </si>
   <si>
     <t xml:space="preserve">Von welchen Verwaltungsbezirken ist Mittelfranken umgeben?</t>
@@ -516,7 +514,7 @@
     <t xml:space="preserve">Welche Bundesländer liegen nördlich von Thüringen?</t>
   </si>
   <si>
-    <t xml:space="preserve">Das Bundesland Thüringen ist mit Hamburg, Schleswig-Holstein, Mecklenburg-Vorpommern, Thüringen und Sachsen-Anhalt verbunden.</t>
+    <t xml:space="preserve">Nördlich des Bundeslands Thüringen liegen Hamburg, Schleswig-Holstein, Mecklenburg-Vorpommern und Sachsen-Anhalt.</t>
   </si>
   <si>
     <t xml:space="preserve">Welche Landkreise liegen westlich vom Landkreis Münster?</t>
@@ -525,28 +523,28 @@
     <t xml:space="preserve">Die Kreise Kleve und Borken liegen westlich von Münster.</t>
   </si>
   <si>
-    <t xml:space="preserve">Welche Verwaltungsgemeinschaften liegen nördlich der Verwaltungsgemeinschaft Morbach?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die nördlich von Morbach gelegenen Gemeinden sind Emlichheim, Viöl, Osterholz-Scharmbeck, Kappeln-Land, Wilster, Vordereifel, Wangerland, Ovelgönne, Schortens, Wangerooge, Südtondern, Brookmerland, Kellinghusen, Cappeln (Oldenburg), Wagenfeld, Mittelholstein, Rendsburg, Wietmarschen, Georgsmarienhütte, Hasbergen, Pinneberg, Marne-Nordsee, Rengsdorf-Waldbreitbach, Bokhorst-Wankendorf, Rantzau, Mittleres Nordfriesland, Hamm (Sieg), Südbrookmerland, Tornesch, Selsingen, Esens, Langeoog, Drochtersen, Glandorf, Elmshorn-Land, Steinfeld (Oldenburg), Lengerich, Steyerberg, Aurich, Bohmte, Bönebüttel, Butjadingen, Geeste, Wasbek, Rehden, Apensen, Stadland, Damme, Bad Essen, Westerstede, Schlei-Ostsee, Westoverledingen, Bad Bentheim, Langballig, Bad Hönningen, Weyhe, Eidertal, Werlte, Elmshorn, Bunde, Horst-Herzhorn, Brunsbüttel, Ihlow, Barßel, Bakum, Garrel, Artland, Tarmstedt, Jever, Landschaft Sylt, Arensharde, Nordhorn, Gnarrenburg, Eiderkanal, Holdorf, Insel Lütje Hörn, Husum, Eiderstedt, Kappeln, Schüttorf, Zell (Mosel), Altenahr, Sylt, Ritterhude, Süderbrarup, Neuenkirchen, Hesel, Wildeshausen, Dänischenhagen, Wurster Nordseeküste, Emsbüren, Fockbek, Vechta, Berne, Nordsee-Treene, Bruchhausen-Vilsen, Kirchspielslandgemeinden Eider, Cochem, Hagen am Teutoburger Wald, Mittelangeln, Hohner Harde, Uelsen, Twistringen, Bramsche, Bad Neuenahr-Ahrweiler, Herzlake, Rhede (Ems), Schrevenborn, Stade, Schwanewede, Wittmund, Borkum, Bad Zwischenahn, Sittensen, Sulingen, Heide, Dötlingen, Glücksburg (Ostsee), Schleswig, Weener, Oeversee, Mendig, Salzbergen, Nordenham, Handewitt, Südangeln, Pinnau, Pellworm, Cuxhaven, Uplengen, Geestequelle, Ottersberg, Kirchdorf, Dinklage, Puderbach, Breitenburg, Nordhümmling, Jümme, Rhauderfehn, Rotenburg (Wümme), Maifeld, Hage, Zeven, Haren (Ems), Sande, Preetz-Land, Wardenburg, Syke, Eggebek, Langwedel, Grafschaft Hoya, Schwentinental, Lemwerder, Jemgum, Barmstedt, Fürstenau, Juist, Visbek, Oldenburg (Oldb), Burg-St. Michaelisdonn, Beverstedt, Lathen, Meppen, Geltinger Bucht, Hilter am Teutoburger Wald, Altenkirchen-Flammersfeld, Lilienthal, Rastede, Adenau, Auenland Südholstein, Uchte, Bissendorf, Flensburg, Kiel, Grasberg, Mitteldithmarschen, Hörnerkirchen, Wiesmoor, Bad Laer, Kaltenkirchen, Altes Amt Lemförde, Barnstorf, Elsfleth, Ostrhauderfehn, Harpstedt, Hatten, Itzehoe, Belm, Bersenbrück, Helgoland, Schenefeld, Neuwied, Andernach, Oldendorf-Himmelpforten, Oyten, Itzehoe-Land, Harrislee, Norden, Kirchspielslandgemeinde Heider Umland, Asbach, Melle, Sögel, Kropp-Stapelholm, Haddeby, Papenburg, Apen, Reußenköge, Fredenbeck, Kelberg, Achterwehr, Siedenburg, Spiekeroog, Bad Rothenfelde, Zetel, Remagen, Baltrum, Neuenkirchen-Vörden, Uetersen, Cloppenburg, Schiffdorf, Linz am Rhein, Leer (Ostfriesland), Wilstermarsch, Ulmen, Dissen am Teutoburger Wald, Schwaförden, Moormerland, Hürup, Emden, Mayen, Großefehn, Unkel, Worpswede, Sinzig, Bösel, Harsefeld, Neumünster, Neuenhaus, Jade, Bad Breisig, Friedrichstadt, Friesoythe, Jork, Hagen im Bremischen, Holtriem, Verden (Aller), Probstei, Lastrup, Sottrum, Lindern (Oldenburg), Ostercappeln, Bad Bramstedt, Dornum, Goldenstedt, Lingen (Ems), Freren, Emstek, Börde Lamstedt, Essen (Oldenburg), Geest und Marsch Südholstein, Schafflund, Bordesholm, Nordseeinsel Memmert, Dänischer Wohld, Saterland, Nortorfer Land, Bockhorn, Geestland, Molbergen, Jevenstedt, Loxstedt, Büdelsdorf, Föhr-Amrum, Krummhörn, Dörpen, Norderney, Bremervörde, Bad Bramstedt-Land, Stuhr, Wilhelmshaven, Tönning, Hemmoor, Haselünne, Wallenhorst, Thedinghausen, Kaisersesch, Kronshagen, Großheide, Friedeburg, Lühe, Brake (Unterweser), Bad Iburg, Traben-Trarbach, Brohltal, Löningen, Grafschaft, Twist, Eckernförde, Pellenz, Ganderkesee, Großenkneten, Krempermarsch, Diepholz, Nordkehdingen, Hude (Oldb), Varel, Altenholz, Delmenhorst, Büsum-Wesselburen, Osnabrück, Hinte, Hambergen, Glückstadt, Wedel, Bassum, Horneburg, Edewecht, Hüttener Berge, Achim, Wiefelstede, Lohne (Oldenburg), Spelle, und Land Hadeln.</t>
+    <t xml:space="preserve">Welche Verwaltungsgemeinschaften liegen nördlich der Verwaltungsgemeinschaft Kiel?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Die nördlich der Verwaltungsgemeinde Kiel gelegenen Verwaltungsgemeinden sind: Altenholz, Dänischenhagen, Kappeln und Geltinger Bucht.</t>
   </si>
   <si>
     <t xml:space="preserve">Welche Landkreise liegen in einem Umkreis von 10 km um den Kreis Göttingen?</t>
   </si>
   <si>
-    <t xml:space="preserve">Der Landkreis Göttingen liegt in einem Umkreis von 10 km um die folgenden Landkreise: Eichsfeld, Werra-Meißner-Kreis, Harz, Kassel, Goslar, Northeim, Nordhausen und Kassel.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welche Städte liegen in einem Umkreis von 15 km um Aachen?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">In einem Umkreis von 15 km um die Stadt Aachen liegen folgende Städte: Stolberg (Rhld.), Aldenhoven, Rötgen, Gangelt, Nideggen, Inden, Eschweiler, Heimbach, Baesweiler, Alsdorf, Linnich, Würselen, Langerwehe, Monschau, Hürtgenwald, Kreuzau, Düren, Jülich, Simmerath, Geilenkirchen, Übach-Palenberg und Herzogenrath.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Welche Städte liegen in einem Umkreis von weniger als 20 km um München?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Die Städte und Orte im Umkreis von weniger als 20 km um München sind: Haar, Forstenrieder Park, Unterföhring, Bergkirchen, Berg, Markt Schwaben, Weichs, Wörth, Starnberg, Neuried, Mammendorf, Sulzemoos, Moorenweis, Hohenkammer, Schöngeising, Schwabhausen, Hohenlinden, Olching, Marzling, Allershausen, Grünwald, Weßling, Alling, Planegg, Putzbrunn, Odelzhausen, Eglhartinger Forst, Oberschleißheim, Poing, Landsberied, Taufkirchen, Vaterstetten, Forstern, Inning a.Ammersee, Wolfratshausen, Münsing, Andechs, Grafrath, Finsing, Kirchseeon, Wörthsee, Petershausen, Fahrenzhausen, Schäftlarn, Krailling, Aschheim, Altomünster, Maisach, Egmating, Karlsfeld, Ebersberg, Ottobrunn, Aying, Röhrmoos, Zorneding, Unterhaching, Haimhausen, Neuching, Kottgeisering, Oberhaching, Erding, Adelshofen, Althegnenberg, Eching am Ammersee, Ismaning, Brunnthal, Forstinning, Walpertskirchen, Bruck, Gröbenzell, Freising, Baierbrunn, Türkenfeld, Egling, Oberding, Aßling, Kirchheim b.München, Garching b.München, Emmering, Otterfing, Germering, Neubiberg, Pliening, Baiern, Eching, Ebersberger Forst, Valley, Kranzberg, Icking, Pfaffenhofen a.d.Glonn, Anzinger Forst, Markt Indersdorf, Vierkirchen, Feldkirchen-Westerham, Jetzendorf, Fürstenfeldbruck, Moosinning, Feldkirchen, Grünwalder Forst, Hallbergmoos, Geretsried, Ammersee, Hebertshausen, Wolfratshauser Forst, Dietramszell, Egenhofen, Starnberger See, Unterschleißheim, Gauting, Neufahrn b.Freising, Straßlach-Dingharting, Perlacher Forst, Höhenkirchen-Siegertsbrunn, Moosach, Dachau, Hattenhofen, Grafing b.München, Pullach i.Isartal, Grasbrunn, Oberpframmern, Ottenhofen, Gilching, Anzing, Pöcking, Mittelstetten, Erdweg, Glonn, Gräfelfing, Holzkirchen, Pupplinger Au, Feldafing, Jesenwang, Pastetten, Sauerlach, Eichenau, Oberschweinbach, Weyarn, Seefeld, Puchheim, Hohenbrunn, and Herrsching a.Ammersee.</t>
+    <t xml:space="preserve">Der Landkreis Göttingen umfasst im Umkreis von 10 km folgende Landkreise: Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis und Nordhausen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welche Städte liegen in einem Umkreis von 5 km um Aachen?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In einem Umkreis von 5 km um die Stadt Aachen liegen folgende Städte: Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen,  Herzogenrath, Eschweiler, Stolberg (Rhld.).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welche Städte liegen in einem Umkreis von weniger als 2 km um München?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zu den Städten, die weniger als 2 km von München entfernt liegen, gehören: Forstenrieder Park, Grünwald, Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i. Isartal, Bergkirchen, Neuried, Germering, Olching, Garching bei München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing und Karlsfeld.</t>
   </si>
   <si>
     <t xml:space="preserve">FR</t>
@@ -561,7 +559,7 @@
     <t xml:space="preserve">Où se trouve la ville de Cologne ?</t>
   </si>
   <si>
-    <t xml:space="preserve">La ville de Cologne s'appelle Köln ; elle est située dans l'arrondissement de Köln, dans la circonscription administrative de Köln et dans le Land de Rhénanie-du-Nord-Westphalie.</t>
+    <t xml:space="preserve">La ville de Cologne est située dans l'arrondissement de Cologne, dans le Land de Rhénanie-du-Nord-Westphalie.</t>
   </si>
   <si>
     <t xml:space="preserve">Où se trouve la communauté de communes d'Eisenhüttenstadt ?</t>
@@ -579,7 +577,7 @@
     <t xml:space="preserve">Où se trouve l'arrondissement de Giessen ?</t>
   </si>
   <si>
-    <t xml:space="preserve">L'arrondissement de Gießen est situé à Gießen, en Hesse. Les niveaux hiérarchiques sont les suivants : arrondissement de Gießen et Land de Hesse.</t>
+    <t xml:space="preserve">L'arrondissement de Giessen est situé dans le Land de Hesse.</t>
   </si>
   <si>
     <t xml:space="preserve">Où se trouve l'arrondissement de Saxe du Nord ?</t>
@@ -603,13 +601,13 @@
     <t xml:space="preserve">Où se trouve le Land de Saxe ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Le Land de Saxe est situé au POINT (13.348518008906732 51.05230081187263).</t>
+    <t xml:space="preserve">Le Land de Saxe se situe au niveau fédéral. Les coordonnées du centre de gravité de la Saxe sont les suivantes : POINT (13,348518008906732 51,05230081187263).</t>
   </si>
   <si>
     <t xml:space="preserve">Où se trouve la Sarre ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Le Land de Sarre se situe au niveau du Land.</t>
+    <t xml:space="preserve">La Sarre est un Land au niveau fédéral. Les coordonnées du centre de gravité de la Sarre sont les suivantes : POINT (6,953360955673903 49,38438040655551).</t>
   </si>
   <si>
     <t xml:space="preserve">Quelles villes font partie de l'arrondissement de Coesfeld ?</t>
@@ -657,7 +655,7 @@
     <t xml:space="preserve">La région administrative de Haute-Franconie fait-elle partie du Land de Bavière ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Oui, le district administratif de Haute-Franconie fait partie du Land de Bavière. Le district administratif est la Haute-Franconie, et le Land est la Bavière.</t>
+    <t xml:space="preserve">Oui, le district administratif de Haute-Franconie fait partie du Land de Bavière.</t>
   </si>
   <si>
     <t xml:space="preserve">L'arrondissement de Steinfurt se trouve-t-il dans le Land de Rhénanie-du-Nord-Westphalie ?</t>
@@ -693,25 +691,25 @@
     <t xml:space="preserve">Berlin est-elle entièrement entourée par le Brandebourg ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Oui.</t>
+    <t xml:space="preserve">Oui, Berlin est entourée par le Brandebourg.</t>
   </si>
   <si>
     <t xml:space="preserve">Münster se trouve-t-elle au nord de Dortmund ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Oui, Münster se trouve au nord de Dortmund. Dortmund est une ville, tout comme Münster.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelle ville se trouve juste au nord de Jever ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Le Wangerland est situé directement au nord de Jever.</t>
+    <t xml:space="preserve">Oui, Münster se trouve au nord de Dortmund.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelle ville se trouve juste au nord de Münster?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le Greven est situé directement au nord de Münster.</t>
   </si>
   <si>
     <t xml:space="preserve">Leipzig se trouve-t-elle à l'est d'Erfurt ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Oui. Leipzig est située au nord-est d’Erfurt.</t>
+    <t xml:space="preserve">Oui, Leipzig est située au nord-est d’Erfurt.</t>
   </si>
   <si>
     <t xml:space="preserve">Quelle est la distance entre Cologne et Bonn ?</t>
@@ -744,10 +742,10 @@
     <t xml:space="preserve">Le district de Warendorf est limitrophe des districts de Gütersloh, Münster, Osnabrück, Steinfurt, Hamm, Coesfeld et Soest.</t>
   </si>
   <si>
-    <t xml:space="preserve">Quelles communautés administratives sont limitrophes de Leezen ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">« Les communes administratives limitrophes de Leezen sont Groß Niendorf, Mözen, Kükels, Fredesdorf, Seth, Sülfeld, Neversdorf et Bebensee. Leezen est également limitrophe de Langen Brütz, Lübstorf, Raben Steinfeld, Cambs, Dobin am See, Schwerin, Gneven et Pinnow.</t>
+    <t xml:space="preserve">Quelles sont les communes administratives limitrophes de la commune administrative de Leezen ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La commune de Leezen est limitrophe des communes suivantes : Auenland Südholstein, Kisdorf, Bad Oldesloe-Land, Trave-Land, Wahlstedt, Itzstedt, Bad Segeberg, Boostedt-Rickling et Buchholz (Forstgutsbez.).</t>
   </si>
   <si>
     <t xml:space="preserve">De quels districts administratifs la Moyenne-Franconie est-elle entourée ?</t>
@@ -759,7 +757,7 @@
     <t xml:space="preserve">Quels sont les Länder situés au nord de la Thuringe ?</t>
   </si>
   <si>
-    <t xml:space="preserve">Le Land de Thuringe est limitrophe de Hambourg, du Schleswig-Holstein, du Mecklembourg-Poméranie occidentale, de la Thuringe et de la Saxe-Anhalt.</t>
+    <t xml:space="preserve">Les Länder situés au nord de la Thuringe sont Hambourg, le Schleswig-Holstein, le Mecklembourg-Poméranie occidentale et la Saxe-Anhalt.</t>
   </si>
   <si>
     <t xml:space="preserve">Quels sont les districts situés à l'ouest de district Münster ?</t>
@@ -768,28 +766,28 @@
     <t xml:space="preserve">Les districts de Clèves et de Borken se trouvent à l'ouest de Münster.</t>
   </si>
   <si>
-    <t xml:space="preserve">Quelles sont les communautés administratives situées au nord de la communauté administrative de Morbach ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Les communes situées au nord de Morbach sont Emlichheim, Viöl, Osterholz-Scharmbeck, Kappeln-Land, Wilster, Vordereifel, Wangerland, Ovelgönne, Schortens, Wangerooge, Südtondern, Brookmerland, Kellinghusen, Cappeln (Oldenburg), Wagenfeld, Mittelholstein, Rendsburg, Wietmarschen, Georgsmarienhütte, Hasbergen, Pinneberg, Marne-Nordsee, Rengsdorf-Waldbreitbach, Bokhorst-Wankendorf, Rantzau, Mittleres Nordfriesland, Hamm (Sieg), Südbrookmerland, Tornesch, Selsingen, Esens, Langeoog, Drochtersen, Glandorf, Elmshorn-Land, Steinfeld (Oldenburg), Lengerich, Steyerberg, Aurich, Bohmte, Bönebüttel, Butjadingen, Geeste, Wasbek, Rehden, Apensen, Stadland, Damme, Bad Essen, Westerstede, Schlei-Ostsee, Westoverledingen, Bad Bentheim, Langballig, Bad Hönningen, Weyhe, Eidertal, Werlte, Elmshorn, Bunde, Horst-Herzhorn, Brunsbüttel, Ihlow, Barßel, Bakum, Garrel, Artland, Tarmstedt, Jever, Landschaft Sylt, Arensharde, Nordhorn, Gnarrenburg, Eiderkanal, Holdorf, Insel Lütje Hörn, Husum, Eiderstedt, Kappeln, Schüttorf, Zell (Mosel), Altenahr, Sylt, Ritterhude, Süderbrarup, Neuenkirchen, Hesel, Wildeshausen, Dänischenhagen, Wurster Nordseeküste, Emsbüren, Fockbek, Vechta, Berne, Nordsee-Treene, Bruchhausen-Vilsen, Kirchspielslandgemeinden Eider, Cochem, Hagen am Teutoburger Wald, Mittelangeln, Hohner Harde, Uelsen, Twistringen, Bramsche, Bad Neuenahr-Ahrweiler, Herzlake, Rhede (Ems), Schrevenborn, Stade, Schwanewede, Wittmund, Borkum, Bad Zwischenahn, Sittensen, Sulingen, Heide, Dötlingen, Glücksburg (Ostsee), Schleswig, Weener, Oeversee, Mendig, Salzbergen, Nordenham, Handewitt, Südangeln, Pinnau, Pellworm, Cuxhaven, Uplengen, Geestequelle, Ottersberg, Kirchdorf, Dinklage, Puderbach, Breitenburg, Nordhümmling, Jümme, Rhauderfehn, Rotenburg (Wümme), Maifeld, Hage, Zeven, Haren (Ems), Sande, Preetz-Land, Wardenburg, Syke, Eggebek, Langwedel, Grafschaft Hoya, Schwentinental, Lemwerder, Jemgum, Barmstedt, Fürstenau, Juist, Visbek, Oldenburg (Oldb), Burg-St. Michaelisdonn, Beverstedt, Lathen, Meppen, Geltinger Bucht, Hilter am Teutoburger Wald, Altenkirchen-Flammersfeld, Lilienthal, Rastede, Adenau, Auenland Südholstein, Uchte, Bissendorf, Flensburg, Kiel, Grasberg, Mitteldithmarschen, Hörnerkirchen, Wiesmoor, Bad Laer, Kaltenkirchen, Altes Amt Lemförde, Barnstorf, Elsfleth, Ostrhauderfehn, Harpstedt, Hatten, Itzehoe, Belm, Bersenbrück, Helgoland, Schenefeld, Neuwied, Andernach, Oldendorf-Himmelpforten, Oyten, Itzehoe-Land, Harrislee, Norden, Kirchspielslandgemeinde Heider Umland, Asbach, Melle, Sögel, Kropp-Stapelholm, Haddeby, Papenburg, Apen, Reußenköge, Fredenbeck, Kelberg, Achterwehr, Siedenburg, Spiekeroog, Bad Rothenfelde, Zetel, Remagen, Baltrum, Neuenkirchen-Vörden, Uetersen, Cloppenburg, Schiffdorf, Linz am Rhein, Leer (Ostfriesland), Wilstermarsch, Ulmen, Dissen am Teutoburger Wald, Schwaförden, Moormerland, Hürup, Emden, Mayen, Großefehn, Unkel, Worpswede, Sinzig, Bösel, Harsefeld, Neumünster, Neuenhaus, Jade, Bad Breisig, Friedrichstadt, Friesoythe, Jork, Hagen im Bremischen, Holtriem, Verden (Aller), Probstei, Lastrup, Sottrum, Lindern (Oldenburg), Ostercappeln, Bad Bramstedt, Dornum, Goldenstedt, Lingen (Ems), Freren, Emstek, Börde Lamstedt, Essen (Oldenburg), Geest und Marsch Südholstein, Schafflund, Bordesholm, Nordseeinsel Memmert, Dänischer Wohld, Saterland, Nortorfer Land, Bockhorn, Geestland, Molbergen, Jevenstedt, Loxstedt, Büdelsdorf, Föhr-Amrum, Krummhörn, Dörpen, Norderney, Bremervörde, Bad Bramstedt-Land, Stuhr, Wilhelmshaven, Tönning, Hemmoor, Haselünne, Wallenhorst, Thedinghausen, Kaisersesch, Kronshagen, Großheide, Friedeburg, Lühe, Brake (Unterweser), Bad Iburg, Traben-Trarbach, Brohltal, Löningen, Grafschaft, Twist, Eckernförde, Pellenz, Ganderkesee, Großenkneten, Krempermarsch, Diepholz, Nordkehdingen, Hude (Oldb), Varel, Altenholz, Delmenhorst, Büsum-Wesselburen, Osnabrück, Hinte, Hambergen, Glückstadt, Wedel, Bassum, Horneburg, Edewecht, Hüttener Berge, Achim, Wiefelstede, Lohne (Oldenburg), Spelle, e Land Hadeln.</t>
+    <t xml:space="preserve">Quelles sont les communautés administratives situées au nord de la communauté administrative de Kiel ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les communes administratives situées au nord de la commune administrative de Kiel sont : Altenholz, Dänischenhagen, Kappeln et Geltinger Bucht.</t>
   </si>
   <si>
     <t xml:space="preserve">Quels sont les districts situés dans un rayon de 10 km autour de district Göttingen ?</t>
   </si>
   <si>
-    <t xml:space="preserve">L'arrondissement de Göttingen est situé dans un rayon de 10 km autour des arrondissements suivants : Eichsfeld, Werra-Meißner-Kreis, Harz, Kassel, Goslar, Northeim, Nordhausen et Kassel.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelles sont les villes situées dans un rayon de 15 km autour d'Aix-la-Chapelle ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dans un rayon de 15 km autour de la ville d'Aix-la-Chapelle, on trouve les villes suivantes : Stolberg (Rhld.), Aldenhoven, Roetgen, Gangelt, Nideggen, Inden, Eschweiler, Heimbach, Baesweiler, Alsdorf, Linnich, Würselen, Langerwehe, Monschau, Hürtgenwald, Kreuzau, Düren, Jülich, Simmerath, Geilenkirchen, Übach-Palenberg et Herzogenrath.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quelles sont les villes situées dans un rayon de moins de 20 km autour de Munich ?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Les villes et localités situées à moins de 20 km de Munich sont : Haar, Forstenrieder Park, Unterföhring, Bergkirchen, Berg, Markt Schwaben, Weichs, Wörth, Starnberg, Neuried, Mammendorf, Sulzemoos, Moorenweis, Hohenkammer, Schöngeising, Schwabhausen, Hohenlinden, Olching, Marzling, Allershausen, Grünwald, Weßling, Alling, Planegg, Putzbrunn, Odelzhausen, Eglhartinger Forst, Oberschleißheim, Poing, Landsberied, Taufkirchen, Vaterstetten, Forstern, Inning a. Ammersee, Wolfratshausen, Münsing, Andechs, Grafrath, Finsing, Kirchseeon, Wörthsee, Petershausen, Fahrenzhausen, Schäftlarn, Krailling, Aschheim, Altomünster, Maisach, Egmating, Karlsfeld, Ebersberg, Ottobrunn, Aying, Röhrmoos, Zorneding, Unterhaching, Haimhausen, Neuching, Kottgeisering, Oberhaching, Erding, Adelshofen, Althegnenberg, Eching am Ammersee, Ismaning, Brunnthal, Forstinning, Walpertskirchen, Bruck, Gröbenzell, Freising, Baierbrunn, Türkenfeld, Egling, Oberding, Aßling, Kirchheim près de Munich, Garching près de Munich, Emmering, Otterfing, Germering, Neubiberg, Pliening, Baiern, Eching, Ebersberger Forst, Valley, Kranzberg, Icking, Pfaffenhofen a.d.Glonn, Anzinger Forst, Markt Indersdorf, Vierkirchen, Feldkirchen-Westerham, Jetzendorf, Fürstenfeldbruck, Moosinning, Feldkirchen, Grünwalder Forst, Hallbergmoos, Geretsried, Ammersee, Hebertshausen, Wolfratshauser Forst, Dietramszell, Egenhofen, Starnberger See, Unterschleißheim, Gauting, Neufahrn près de Freising, Straßlach-Dingharting, Perlacher Forst, Höhenkirchen-Siegertsbrunn, Moosach, Dachau, Hattenhofen, Grafing près de Munich, Pullach dans la vallée de l'Isar, Grasbrunn, Oberpframmern, Ottenhofen, Gilching, Anzing, Pöcking, Mittelstetten, Erdweg, Glonn, Gräfelfing, Holzkirchen, Pupplinger Au, Feldafing, Jesenwang, Pastetten, Sauerlach, Eichenau, Oberschweinbach, Weyarn, Seefeld, Puchheim, Hohenbrunn et Herrsching a. Ammersee. Toutes ces localités sont répertoriées comme des entités municipales situées autour de Munich, qui est la ville faisant l'objet de la requête.</t>
+    <t xml:space="preserve">Le district de Göttingen comprend les districts suivants dans un rayon de 10 km : Harz, Northeim, Goslar, Kassel, Eichsfeld, Werra-Meißner-Kreis et Nordhausen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelles sont les villes situées dans un rayon de 5 km autour d'Aix-la-Chapelle ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les villes suivantes sont situées dans un rayon de 5 km autour d'Aix-la-Chapelle : Alsdorf, Simmerath, Würselen, Hürtgenwald, Roetgen, Herzogenrath, Eschweiler, Stolberg (Rhld.).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quelles sont les villes situées dans un rayon de moins de 2 km autour de Munich ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les villes situées à moins de 2 km de Munich sont : Forstenrieder Park, Grünwald, Feldkirchen, Aschheim, Haar, Unterhaching, Pullach i.Isartal, Bergkirchen, Neuried, Germering, Olching, Garching b.München, Planegg, Ismaning, Puchheim, Unterföhring, Gröbenzell, Neubiberg, Oberschleißheim, Putzbrunn, Perlacher Forst, Gräfelfing et Karlsfeld.</t>
   </si>
 </sst>
 </file>
@@ -901,7 +899,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -926,6 +924,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -948,7 +950,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D121"/>
-  <sheetFormatPr defaultColWidth="10.5625" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5234375" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="36.05"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.75"/>
@@ -1128,7 +1130,7 @@
       <c r="A13" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C13" s="0" t="s">
@@ -1142,7 +1144,7 @@
       <c r="A14" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C14" s="0" t="s">
@@ -1156,7 +1158,7 @@
       <c r="A15" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C15" s="0" t="s">
@@ -1170,7 +1172,7 @@
       <c r="A16" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="0" t="s">
@@ -1184,7 +1186,7 @@
       <c r="A17" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C17" s="0" t="s">
@@ -1198,7 +1200,7 @@
       <c r="A18" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C18" s="0" t="s">
@@ -1212,7 +1214,7 @@
       <c r="A19" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C19" s="0" t="s">
@@ -1226,7 +1228,7 @@
       <c r="A20" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C20" s="0" t="s">
@@ -1240,7 +1242,7 @@
       <c r="A21" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C21" s="0" t="s">
@@ -1418,14 +1420,14 @@
         <v>75</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="138.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="15.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
         <v>4</v>
       </c>
       <c r="B34" s="0" t="s">
         <v>71</v>
       </c>
-      <c r="C34" s="0" t="s">
+      <c r="C34" s="6" t="s">
         <v>76</v>
       </c>
       <c r="D34" s="6" t="s">
@@ -1502,7 +1504,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="13.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
         <v>4</v>
       </c>
@@ -1516,7 +1518,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="539.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="13.85" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
         <v>4</v>
       </c>
@@ -1526,7 +1528,7 @@
       <c r="C41" s="0" t="s">
         <v>92</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="D41" s="7" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1674,7 +1676,7 @@
       <c r="A52" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B52" s="0" t="s">
+      <c r="B52" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C52" s="0" t="s">
@@ -1688,7 +1690,7 @@
       <c r="A53" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B53" s="0" t="s">
+      <c r="B53" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C53" s="0" t="s">
@@ -1702,7 +1704,7 @@
       <c r="A54" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B54" s="0" t="s">
+      <c r="B54" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C54" s="0" t="s">
@@ -1716,7 +1718,7 @@
       <c r="A55" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B55" s="0" t="s">
+      <c r="B55" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C55" s="0" t="s">
@@ -1730,7 +1732,7 @@
       <c r="A56" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B56" s="0" t="s">
+      <c r="B56" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C56" s="0" t="s">
@@ -1744,7 +1746,7 @@
       <c r="A57" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B57" s="0" t="s">
+      <c r="B57" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C57" s="0" t="s">
@@ -1758,7 +1760,7 @@
       <c r="A58" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B58" s="0" t="s">
+      <c r="B58" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C58" s="0" t="s">
@@ -1772,7 +1774,7 @@
       <c r="A59" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B59" s="0" t="s">
+      <c r="B59" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C59" s="0" t="s">
@@ -1786,7 +1788,7 @@
       <c r="A60" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B60" s="0" t="s">
+      <c r="B60" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C60" s="0" t="s">
@@ -1800,7 +1802,7 @@
       <c r="A61" s="0" t="s">
         <v>94</v>
       </c>
-      <c r="B61" s="0" t="s">
+      <c r="B61" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C61" s="0" t="s">
@@ -2234,7 +2236,7 @@
       <c r="A92" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B92" s="0" t="s">
+      <c r="B92" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C92" s="0" t="s">
@@ -2248,7 +2250,7 @@
       <c r="A93" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B93" s="0" t="s">
+      <c r="B93" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C93" s="0" t="s">
@@ -2262,7 +2264,7 @@
       <c r="A94" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B94" s="0" t="s">
+      <c r="B94" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C94" s="0" t="s">
@@ -2276,7 +2278,7 @@
       <c r="A95" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B95" s="0" t="s">
+      <c r="B95" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C95" s="0" t="s">
@@ -2290,7 +2292,7 @@
       <c r="A96" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B96" s="0" t="s">
+      <c r="B96" s="4" t="s">
         <v>26</v>
       </c>
       <c r="C96" s="0" t="s">
@@ -2304,7 +2306,7 @@
       <c r="A97" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B97" s="0" t="s">
+      <c r="B97" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C97" s="0" t="s">
@@ -2318,7 +2320,7 @@
       <c r="A98" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B98" s="0" t="s">
+      <c r="B98" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C98" s="0" t="s">
@@ -2332,7 +2334,7 @@
       <c r="A99" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B99" s="0" t="s">
+      <c r="B99" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C99" s="0" t="s">
@@ -2346,7 +2348,7 @@
       <c r="A100" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B100" s="0" t="s">
+      <c r="B100" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C100" s="0" t="s">
@@ -2360,7 +2362,7 @@
       <c r="A101" s="0" t="s">
         <v>175</v>
       </c>
-      <c r="B101" s="0" t="s">
+      <c r="B101" s="4" t="s">
         <v>37</v>
       </c>
       <c r="C101" s="0" t="s">

</xml_diff>